<commit_message>
Delay calculations are correct.
</commit_message>
<xml_diff>
--- a/angle.xlsx
+++ b/angle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\radio-zcu208\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E073F8-15C0-47CA-870F-06F0D51839DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110D5E8C-C0E4-4AFF-908B-3BC8D400B257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5760" yWindow="390" windowWidth="19140" windowHeight="10635" xr2:uid="{95DD9B03-E977-4F2B-8BD5-666F9F270815}"/>
+    <workbookView xWindow="2715" yWindow="5205" windowWidth="19140" windowHeight="10635" xr2:uid="{95DD9B03-E977-4F2B-8BD5-666F9F270815}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="28">
   <si>
     <t>EW</t>
   </si>
@@ -111,6 +111,15 @@
   </si>
   <si>
     <t>N</t>
+  </si>
+  <si>
+    <t>Phase</t>
+  </si>
+  <si>
+    <t>Delay</t>
+  </si>
+  <si>
+    <t>Rel</t>
   </si>
 </sst>
 </file>
@@ -497,7 +506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20B124CC-6FFE-47E0-8DD9-E7CCDFA2FBAF}">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="17" customWidth="1"/>
@@ -505,97 +514,97 @@
     <col min="9" max="9" width="10.5703125" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" customWidth="1"/>
     <col min="11" max="13" width="9.5703125" customWidth="1"/>
-    <col min="14" max="14" width="12.28515625" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" customWidth="1"/>
+    <col min="15" max="15" width="8.42578125" customWidth="1"/>
+    <col min="16" max="17" width="8.140625" customWidth="1"/>
+    <col min="18" max="19" width="8" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="O1" t="s">
+        <v>25</v>
+      </c>
+      <c r="R1" t="s">
+        <v>26</v>
+      </c>
+      <c r="U1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F2" t="s">
         <v>3</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H2" t="s">
         <v>17</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I2" t="s">
         <v>18</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J2" t="s">
         <v>15</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K2" t="s">
         <v>16</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L2" t="s">
         <v>19</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>0</v>
-      </c>
-      <c r="B2">
+      <c r="N2" t="s">
+        <v>1</v>
+      </c>
+      <c r="O2" t="s">
+        <v>0</v>
+      </c>
+      <c r="P2" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>1</v>
+      </c>
+      <c r="R2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S2" t="s">
+        <v>2</v>
+      </c>
+      <c r="T2" t="s">
+        <v>1</v>
+      </c>
+      <c r="U2" t="s">
+        <v>0</v>
+      </c>
+      <c r="V2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
         <v>-60</v>
       </c>
-      <c r="C2" s="1">
-        <v>0</v>
-      </c>
-      <c r="D2" s="1">
+      <c r="C3" s="1">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1">
         <v>60</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2">
-        <v>1</v>
-      </c>
-      <c r="I2">
-        <v>0</v>
-      </c>
-      <c r="J2">
-        <v>0</v>
-      </c>
-      <c r="K2">
-        <v>0</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3">
-        <v>10</v>
-      </c>
-      <c r="B3" s="1">
-        <v>-50</v>
-      </c>
-      <c r="C3" s="1">
-        <v>-10</v>
-      </c>
-      <c r="D3">
-        <v>70</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>0</v>
@@ -604,7 +613,7 @@
         <v>5</v>
       </c>
       <c r="G3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -613,30 +622,60 @@
         <v>0</v>
       </c>
       <c r="J3">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3">
+        <v>-278705</v>
+      </c>
+      <c r="O3">
+        <v>0</v>
+      </c>
+      <c r="P3">
+        <v>278705</v>
+      </c>
+      <c r="Q3">
+        <v>-227023</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>227023</v>
+      </c>
+      <c r="T3">
+        <f>N3/Q3</f>
+        <v>1.2276509428560103</v>
+      </c>
+      <c r="U3" s="1" t="e">
+        <f>O3/R3</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V3">
+        <f>P3/S3</f>
+        <v>1.2276509428560103</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1">
-        <v>-40</v>
+        <v>-50</v>
       </c>
       <c r="C4" s="1">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="D4">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>0</v>
@@ -648,36 +687,66 @@
         <v>12</v>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I4">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="J4">
+        <v>-10</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>10</v>
+      </c>
+      <c r="M4" t="s">
+        <v>21</v>
+      </c>
+      <c r="N4">
+        <v>-246525</v>
+      </c>
+      <c r="O4">
+        <v>-55888</v>
+      </c>
+      <c r="P4">
+        <v>302412</v>
+      </c>
+      <c r="Q4">
+        <v>-200800</v>
+      </c>
+      <c r="R4">
+        <v>-45542</v>
+      </c>
+      <c r="S4">
+        <v>246342</v>
+      </c>
+      <c r="T4">
+        <f t="shared" ref="T4:V4" si="0">N4/Q4</f>
+        <v>1.2277141434262948</v>
+      </c>
+      <c r="U4" s="1">
+        <f t="shared" si="0"/>
+        <v>1.2271749154626499</v>
+      </c>
+      <c r="V4">
+        <f t="shared" si="0"/>
+        <v>1.2276103953040893</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1">
         <v>-40</v>
       </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="L4">
-        <v>20</v>
-      </c>
-      <c r="M4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>30</v>
-      </c>
-      <c r="B5" s="1">
-        <v>-30</v>
-      </c>
       <c r="C5" s="1">
-        <v>-30</v>
+        <v>-20</v>
       </c>
       <c r="D5">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>0</v>
@@ -695,39 +764,69 @@
         <v>60</v>
       </c>
       <c r="J5">
-        <v>-30</v>
+        <v>-40</v>
       </c>
       <c r="K5">
         <v>1</v>
       </c>
       <c r="L5">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="M5" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N5">
+        <v>-206860</v>
+      </c>
+      <c r="O5">
+        <v>-110077</v>
+      </c>
+      <c r="P5">
+        <v>316935</v>
+      </c>
+      <c r="Q5">
+        <v>-168579</v>
+      </c>
+      <c r="R5">
+        <v>-89565</v>
+      </c>
+      <c r="S5">
+        <v>258143</v>
+      </c>
+      <c r="T5">
+        <f t="shared" ref="T5" si="1">N5/Q5</f>
+        <v>1.2270804785886735</v>
+      </c>
+      <c r="U5" s="1">
+        <f t="shared" ref="U5:U38" si="2">O5/R5</f>
+        <v>1.2290180315971642</v>
+      </c>
+      <c r="V5">
+        <f t="shared" ref="V5:V38" si="3">P5/S5</f>
+        <v>1.2277497356116571</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="C6" s="1">
-        <v>-40</v>
+        <v>-30</v>
       </c>
       <c r="D6">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -736,30 +835,60 @@
         <v>60</v>
       </c>
       <c r="J6">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="K6">
         <v>1</v>
       </c>
       <c r="L6">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="M6" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6">
+        <v>-160913</v>
+      </c>
+      <c r="O6">
+        <v>-160920</v>
+      </c>
+      <c r="P6">
+        <v>321803</v>
+      </c>
+      <c r="Q6">
+        <v>-131137</v>
+      </c>
+      <c r="R6">
+        <v>-131006</v>
+      </c>
+      <c r="S6">
+        <v>262144</v>
+      </c>
+      <c r="T6" s="1">
+        <f t="shared" ref="T6:T7" si="4">N6/Q6</f>
+        <v>1.2270602499675911</v>
+      </c>
+      <c r="U6">
+        <f t="shared" si="2"/>
+        <v>1.228340686686106</v>
+      </c>
+      <c r="V6">
+        <f t="shared" si="3"/>
+        <v>1.2275810241699219</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B7" s="1">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="C7" s="1">
-        <v>-50</v>
+        <v>-40</v>
       </c>
       <c r="D7">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>1</v>
@@ -777,30 +906,60 @@
         <v>60</v>
       </c>
       <c r="J7">
+        <v>-20</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>40</v>
+      </c>
+      <c r="M7" t="s">
+        <v>22</v>
+      </c>
+      <c r="N7">
+        <v>-110075</v>
+      </c>
+      <c r="O7">
+        <v>-206868</v>
+      </c>
+      <c r="P7">
+        <v>316941</v>
+      </c>
+      <c r="Q7">
+        <v>-89711</v>
+      </c>
+      <c r="R7">
+        <v>-168460</v>
+      </c>
+      <c r="S7">
+        <v>258172</v>
+      </c>
+      <c r="T7" s="1">
+        <f t="shared" si="4"/>
+        <v>1.2269955746786905</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="2"/>
+        <v>1.2279947762080019</v>
+      </c>
+      <c r="V7">
+        <f t="shared" si="3"/>
+        <v>1.2276350649954293</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>50</v>
+      </c>
+      <c r="B8" s="1">
         <v>-10</v>
       </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="L7">
-        <v>50</v>
-      </c>
-      <c r="M7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>60</v>
-      </c>
-      <c r="B8" s="1">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>-60</v>
-      </c>
-      <c r="D8" s="1">
-        <v>60</v>
+      <c r="C8" s="1">
+        <v>-50</v>
+      </c>
+      <c r="D8">
+        <v>70</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>1</v>
@@ -809,7 +968,7 @@
         <v>8</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -818,30 +977,60 @@
         <v>60</v>
       </c>
       <c r="J8">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="K8">
         <v>1</v>
       </c>
       <c r="L8">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N8">
+        <v>-55884</v>
+      </c>
+      <c r="O8">
+        <v>-246534</v>
+      </c>
+      <c r="P8">
+        <v>302417</v>
+      </c>
+      <c r="Q8">
+        <v>-45542</v>
+      </c>
+      <c r="R8">
+        <v>-200800</v>
+      </c>
+      <c r="S8">
+        <v>246342</v>
+      </c>
+      <c r="T8" s="1">
+        <f t="shared" ref="T8:V38" si="5">N8/Q8</f>
+        <v>1.2270870844495192</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="2"/>
+        <v>1.2277589641434263</v>
+      </c>
+      <c r="V8">
+        <f t="shared" si="3"/>
+        <v>1.2276306922895812</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="B9" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="C9">
-        <v>-70</v>
+        <v>-60</v>
       </c>
       <c r="D9" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>1</v>
@@ -859,30 +1048,60 @@
         <v>60</v>
       </c>
       <c r="J9">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K9">
         <v>1</v>
       </c>
       <c r="L9">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="M9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>-278713</v>
+      </c>
+      <c r="P9">
+        <v>278713</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>-227023</v>
+      </c>
+      <c r="S9">
+        <v>227023</v>
+      </c>
+      <c r="T9" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U9">
+        <f t="shared" si="2"/>
+        <v>1.227686181576316</v>
+      </c>
+      <c r="V9">
+        <f t="shared" si="3"/>
+        <v>1.227686181576316</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="B10" s="1">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C10">
-        <v>-80</v>
+        <v>-70</v>
       </c>
       <c r="D10" s="1">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>1</v>
@@ -900,30 +1119,60 @@
         <v>60</v>
       </c>
       <c r="J10">
+        <v>10</v>
+      </c>
+      <c r="K10">
+        <v>1</v>
+      </c>
+      <c r="L10">
+        <v>70</v>
+      </c>
+      <c r="M10" t="s">
+        <v>21</v>
+      </c>
+      <c r="N10">
+        <v>55884</v>
+      </c>
+      <c r="O10">
+        <v>-302417</v>
+      </c>
+      <c r="P10">
+        <v>246534</v>
+      </c>
+      <c r="Q10">
+        <v>45538</v>
+      </c>
+      <c r="R10">
+        <v>-246340</v>
+      </c>
+      <c r="S10">
+        <v>200802</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="5"/>
+        <v>1.2271948702182793</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="2"/>
+        <v>1.2276406592514411</v>
+      </c>
+      <c r="V10">
+        <f t="shared" si="3"/>
+        <v>1.2277467355902829</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>80</v>
+      </c>
+      <c r="B11" s="1">
         <v>20</v>
       </c>
-      <c r="K10">
-        <v>1</v>
-      </c>
-      <c r="L10">
-        <v>80</v>
-      </c>
-      <c r="M10" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <v>90</v>
-      </c>
-      <c r="B11" s="1">
-        <v>30</v>
-      </c>
       <c r="C11">
-        <v>-90</v>
+        <v>-80</v>
       </c>
       <c r="D11" s="1">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>1</v>
@@ -941,39 +1190,69 @@
         <v>60</v>
       </c>
       <c r="J11">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="M11" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N11">
+        <v>110075</v>
+      </c>
+      <c r="O11">
+        <v>-316941</v>
+      </c>
+      <c r="P11">
+        <v>206868</v>
+      </c>
+      <c r="Q11">
+        <v>89705</v>
+      </c>
+      <c r="R11">
+        <v>-258169</v>
+      </c>
+      <c r="S11">
+        <v>168465</v>
+      </c>
+      <c r="T11">
+        <f t="shared" si="5"/>
+        <v>1.2270776433866564</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="2"/>
+        <v>1.2276493304773231</v>
+      </c>
+      <c r="V11">
+        <f t="shared" si="3"/>
+        <v>1.2279583296233638</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B12" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="C12">
-        <v>-80</v>
+        <v>-90</v>
       </c>
       <c r="D12" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F12" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -982,30 +1261,60 @@
         <v>60</v>
       </c>
       <c r="J12">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K12">
         <v>1</v>
       </c>
       <c r="L12">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="M12" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N12">
+        <v>160913</v>
+      </c>
+      <c r="O12">
+        <v>-321803</v>
+      </c>
+      <c r="P12">
+        <v>160920</v>
+      </c>
+      <c r="Q12">
+        <v>131129</v>
+      </c>
+      <c r="R12">
+        <v>-262143</v>
+      </c>
+      <c r="S12">
+        <v>131015</v>
+      </c>
+      <c r="T12">
+        <f t="shared" si="5"/>
+        <v>1.2271351112263496</v>
+      </c>
+      <c r="U12">
+        <f t="shared" si="2"/>
+        <v>1.2275857070377618</v>
+      </c>
+      <c r="V12" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2282563065297867</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="B13" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="C13">
-        <v>-70</v>
+        <v>-80</v>
       </c>
       <c r="D13" s="1">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>2</v>
@@ -1017,36 +1326,66 @@
         <v>11</v>
       </c>
       <c r="H13">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>120</v>
+        <v>60</v>
       </c>
       <c r="J13">
+        <v>40</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>100</v>
+      </c>
+      <c r="M13" t="s">
+        <v>22</v>
+      </c>
+      <c r="N13">
+        <v>206860</v>
+      </c>
+      <c r="O13">
+        <v>-316935</v>
+      </c>
+      <c r="P13">
+        <v>110077</v>
+      </c>
+      <c r="Q13">
+        <v>168568</v>
+      </c>
+      <c r="R13">
+        <v>-258146</v>
+      </c>
+      <c r="S13">
+        <v>89577</v>
+      </c>
+      <c r="T13">
+        <f t="shared" si="5"/>
+        <v>1.2271605524180154</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="2"/>
+        <v>1.2277354675261287</v>
+      </c>
+      <c r="V13" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2288533887046897</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>110</v>
+      </c>
+      <c r="B14" s="1">
+        <v>50</v>
+      </c>
+      <c r="C14">
+        <v>-70</v>
+      </c>
+      <c r="D14" s="1">
         <v>10</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>110</v>
-      </c>
-      <c r="M13" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14">
-        <v>120</v>
-      </c>
-      <c r="B14" s="1">
-        <v>60</v>
-      </c>
-      <c r="C14">
-        <v>-60</v>
-      </c>
-      <c r="D14" s="1">
-        <v>0</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>2</v>
@@ -1064,30 +1403,60 @@
         <v>120</v>
       </c>
       <c r="J14">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K14">
         <v>0</v>
       </c>
       <c r="L14">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="M14" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N14">
+        <v>246525</v>
+      </c>
+      <c r="O14">
+        <v>-302412</v>
+      </c>
+      <c r="P14">
+        <v>55888</v>
+      </c>
+      <c r="Q14">
+        <v>200803</v>
+      </c>
+      <c r="R14">
+        <v>-246341</v>
+      </c>
+      <c r="S14">
+        <v>45537</v>
+      </c>
+      <c r="T14">
+        <f t="shared" si="5"/>
+        <v>1.2276958013575494</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="2"/>
+        <v>1.2276153786823956</v>
+      </c>
+      <c r="V14" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2273096602762588</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>130</v>
-      </c>
-      <c r="B15">
-        <v>70</v>
-      </c>
-      <c r="C15" s="1">
-        <v>-50</v>
+        <v>120</v>
+      </c>
+      <c r="B15" s="1">
+        <v>60</v>
+      </c>
+      <c r="C15">
+        <v>-60</v>
       </c>
       <c r="D15" s="1">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>2</v>
@@ -1096,7 +1465,7 @@
         <v>6</v>
       </c>
       <c r="G15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H15">
         <v>2</v>
@@ -1105,30 +1474,60 @@
         <v>120</v>
       </c>
       <c r="J15">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K15">
         <v>0</v>
       </c>
       <c r="L15">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="M15" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N15">
+        <v>278705</v>
+      </c>
+      <c r="O15">
+        <v>-278705</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>227023</v>
+      </c>
+      <c r="R15">
+        <v>-227023</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <f t="shared" si="5"/>
+        <v>1.2276509428560103</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="2"/>
+        <v>1.2276509428560103</v>
+      </c>
+      <c r="V15" s="1" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="B16">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C16" s="1">
-        <v>-40</v>
+        <v>-50</v>
       </c>
       <c r="D16" s="1">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>2</v>
@@ -1140,36 +1539,66 @@
         <v>12</v>
       </c>
       <c r="H16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="J16">
+        <v>-10</v>
+      </c>
+      <c r="K16">
+        <v>0</v>
+      </c>
+      <c r="L16">
+        <v>130</v>
+      </c>
+      <c r="M16" t="s">
+        <v>21</v>
+      </c>
+      <c r="N16">
+        <v>302412</v>
+      </c>
+      <c r="O16">
+        <v>-246525</v>
+      </c>
+      <c r="P16">
+        <v>-55888</v>
+      </c>
+      <c r="Q16">
+        <v>246342</v>
+      </c>
+      <c r="R16">
+        <v>-200800</v>
+      </c>
+      <c r="S16">
+        <v>-45542</v>
+      </c>
+      <c r="T16">
+        <f t="shared" si="5"/>
+        <v>1.2276103953040893</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="2"/>
+        <v>1.2277141434262948</v>
+      </c>
+      <c r="V16" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2271749154626499</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>140</v>
+      </c>
+      <c r="B17">
+        <v>80</v>
+      </c>
+      <c r="C17" s="1">
         <v>-40</v>
       </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16">
-        <v>140</v>
-      </c>
-      <c r="M16" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17">
-        <v>150</v>
-      </c>
-      <c r="B17">
-        <v>90</v>
-      </c>
-      <c r="C17" s="1">
-        <v>-30</v>
-      </c>
       <c r="D17" s="1">
-        <v>-30</v>
+        <v>-20</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>2</v>
@@ -1187,39 +1616,69 @@
         <v>180</v>
       </c>
       <c r="J17">
-        <v>-30</v>
+        <v>-40</v>
       </c>
       <c r="K17">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L17">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="M17" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N17">
+        <v>316935</v>
+      </c>
+      <c r="O17">
+        <v>-206860</v>
+      </c>
+      <c r="P17">
+        <v>-110077</v>
+      </c>
+      <c r="Q17">
+        <v>258143</v>
+      </c>
+      <c r="R17">
+        <v>-168579</v>
+      </c>
+      <c r="S17">
+        <v>-89565</v>
+      </c>
+      <c r="T17">
+        <f t="shared" si="5"/>
+        <v>1.2277497356116571</v>
+      </c>
+      <c r="U17">
+        <f t="shared" si="2"/>
+        <v>1.2270804785886735</v>
+      </c>
+      <c r="V17" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2290180315971642</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="B18">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="C18" s="1">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="D18" s="1">
-        <v>-40</v>
+        <v>-30</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F18" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G18" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H18">
         <v>1</v>
@@ -1228,30 +1687,60 @@
         <v>180</v>
       </c>
       <c r="J18">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="K18">
         <v>1</v>
       </c>
       <c r="L18">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="M18" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N18">
+        <v>321803</v>
+      </c>
+      <c r="O18">
+        <v>-160913</v>
+      </c>
+      <c r="P18">
+        <v>-160920</v>
+      </c>
+      <c r="Q18">
+        <v>262144</v>
+      </c>
+      <c r="R18">
+        <v>-131137</v>
+      </c>
+      <c r="S18">
+        <v>-131006</v>
+      </c>
+      <c r="T18">
+        <f t="shared" si="5"/>
+        <v>1.2275810241699219</v>
+      </c>
+      <c r="U18" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2270602499675911</v>
+      </c>
+      <c r="V18">
+        <f t="shared" si="3"/>
+        <v>1.228340686686106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B19">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="C19" s="1">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="D19" s="1">
-        <v>-50</v>
+        <v>-40</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>0</v>
@@ -1269,30 +1758,60 @@
         <v>180</v>
       </c>
       <c r="J19">
+        <v>-20</v>
+      </c>
+      <c r="K19">
+        <v>1</v>
+      </c>
+      <c r="L19">
+        <v>160</v>
+      </c>
+      <c r="M19" t="s">
+        <v>24</v>
+      </c>
+      <c r="N19">
+        <v>316941</v>
+      </c>
+      <c r="O19">
+        <v>-110075</v>
+      </c>
+      <c r="P19">
+        <v>-206868</v>
+      </c>
+      <c r="Q19">
+        <v>258172</v>
+      </c>
+      <c r="R19">
+        <v>-89711</v>
+      </c>
+      <c r="S19">
+        <v>-168460</v>
+      </c>
+      <c r="T19">
+        <f t="shared" si="5"/>
+        <v>1.2276350649954293</v>
+      </c>
+      <c r="U19" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2269955746786905</v>
+      </c>
+      <c r="V19">
+        <f t="shared" si="3"/>
+        <v>1.2279947762080019</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>170</v>
+      </c>
+      <c r="B20">
+        <v>70</v>
+      </c>
+      <c r="C20" s="1">
         <v>-10</v>
       </c>
-      <c r="K19">
-        <v>1</v>
-      </c>
-      <c r="L19">
-        <v>170</v>
-      </c>
-      <c r="M19" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20">
-        <v>180</v>
-      </c>
-      <c r="B20" s="1">
-        <v>60</v>
-      </c>
-      <c r="C20" s="1">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>-60</v>
+      <c r="D20" s="1">
+        <v>-50</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>0</v>
@@ -1301,7 +1820,7 @@
         <v>9</v>
       </c>
       <c r="G20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H20">
         <v>1</v>
@@ -1310,30 +1829,60 @@
         <v>180</v>
       </c>
       <c r="J20">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="K20">
         <v>1</v>
       </c>
       <c r="L20">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="M20" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N20">
+        <v>302417</v>
+      </c>
+      <c r="O20">
+        <v>-55884</v>
+      </c>
+      <c r="P20">
+        <v>-246534</v>
+      </c>
+      <c r="Q20">
+        <v>246342</v>
+      </c>
+      <c r="R20">
+        <v>-45542</v>
+      </c>
+      <c r="S20">
+        <v>-200800</v>
+      </c>
+      <c r="T20">
+        <f t="shared" si="5"/>
+        <v>1.2276306922895812</v>
+      </c>
+      <c r="U20" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2270870844495192</v>
+      </c>
+      <c r="V20">
+        <f t="shared" si="3"/>
+        <v>1.2277589641434263</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="B21" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="C21" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="D21">
-        <v>-70</v>
+        <v>-60</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>0</v>
@@ -1351,30 +1900,60 @@
         <v>180</v>
       </c>
       <c r="J21">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K21">
         <v>1</v>
       </c>
       <c r="L21">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="M21" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N21">
+        <v>278713</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>-278713</v>
+      </c>
+      <c r="Q21">
+        <v>227023</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>-227023</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="5"/>
+        <v>1.227686181576316</v>
+      </c>
+      <c r="U21" s="1" t="e">
+        <f t="shared" si="2"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="V21">
+        <f t="shared" si="3"/>
+        <v>1.227686181576316</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="B22" s="1">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C22" s="1">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D22">
-        <v>-80</v>
+        <v>-70</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>0</v>
@@ -1392,30 +1971,60 @@
         <v>180</v>
       </c>
       <c r="J22">
+        <v>10</v>
+      </c>
+      <c r="K22">
+        <v>1</v>
+      </c>
+      <c r="L22">
+        <v>190</v>
+      </c>
+      <c r="M22" t="s">
+        <v>21</v>
+      </c>
+      <c r="N22">
+        <v>246534</v>
+      </c>
+      <c r="O22">
+        <v>55884</v>
+      </c>
+      <c r="P22">
+        <v>-302417</v>
+      </c>
+      <c r="Q22">
+        <v>200802</v>
+      </c>
+      <c r="R22">
+        <v>45538</v>
+      </c>
+      <c r="S22">
+        <v>-246340</v>
+      </c>
+      <c r="T22">
+        <f t="shared" si="5"/>
+        <v>1.2277467355902829</v>
+      </c>
+      <c r="U22" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2271948702182793</v>
+      </c>
+      <c r="V22">
+        <f t="shared" si="3"/>
+        <v>1.2276406592514411</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>200</v>
+      </c>
+      <c r="B23" s="1">
+        <v>40</v>
+      </c>
+      <c r="C23" s="1">
         <v>20</v>
       </c>
-      <c r="K22">
-        <v>1</v>
-      </c>
-      <c r="L22">
-        <v>200</v>
-      </c>
-      <c r="M22" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23">
-        <v>210</v>
-      </c>
-      <c r="B23" s="1">
-        <v>30</v>
-      </c>
-      <c r="C23" s="1">
-        <v>30</v>
-      </c>
       <c r="D23">
-        <v>-90</v>
+        <v>-80</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>0</v>
@@ -1433,39 +2042,69 @@
         <v>180</v>
       </c>
       <c r="J23">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K23">
         <v>1</v>
       </c>
       <c r="L23">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="M23" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N23">
+        <v>206868</v>
+      </c>
+      <c r="O23">
+        <v>110075</v>
+      </c>
+      <c r="P23">
+        <v>-316941</v>
+      </c>
+      <c r="Q23">
+        <v>168465</v>
+      </c>
+      <c r="R23">
+        <v>89705</v>
+      </c>
+      <c r="S23">
+        <v>-258169</v>
+      </c>
+      <c r="T23">
+        <f t="shared" si="5"/>
+        <v>1.2279583296233638</v>
+      </c>
+      <c r="U23" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2270776433866564</v>
+      </c>
+      <c r="V23">
+        <f t="shared" si="3"/>
+        <v>1.2276493304773231</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="B24" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C24" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D24">
-        <v>-80</v>
+        <v>-90</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F24" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G24" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H24">
         <v>1</v>
@@ -1474,30 +2113,60 @@
         <v>180</v>
       </c>
       <c r="J24">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K24">
         <v>1</v>
       </c>
       <c r="L24">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="M24" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N24">
+        <v>160920</v>
+      </c>
+      <c r="O24">
+        <v>160913</v>
+      </c>
+      <c r="P24">
+        <v>-321830</v>
+      </c>
+      <c r="Q24">
+        <v>131015</v>
+      </c>
+      <c r="R24">
+        <v>131129</v>
+      </c>
+      <c r="S24">
+        <v>-262143</v>
+      </c>
+      <c r="T24">
+        <f t="shared" si="5"/>
+        <v>1.2282563065297867</v>
+      </c>
+      <c r="U24" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2271351112263496</v>
+      </c>
+      <c r="V24">
+        <f t="shared" si="3"/>
+        <v>1.227688704256837</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="B25" s="1">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C25" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D25">
-        <v>-70</v>
+        <v>-80</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>1</v>
@@ -1509,36 +2178,66 @@
         <v>11</v>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I25">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="J25">
+        <v>40</v>
+      </c>
+      <c r="K25">
+        <v>1</v>
+      </c>
+      <c r="L25">
+        <v>220</v>
+      </c>
+      <c r="M25" t="s">
+        <v>24</v>
+      </c>
+      <c r="N25">
+        <v>110077</v>
+      </c>
+      <c r="O25">
+        <v>206860</v>
+      </c>
+      <c r="P25">
+        <v>-316935</v>
+      </c>
+      <c r="Q25">
+        <v>89578</v>
+      </c>
+      <c r="R25">
+        <v>168568</v>
+      </c>
+      <c r="S25">
+        <v>-258146</v>
+      </c>
+      <c r="T25" s="1">
+        <f t="shared" si="5"/>
+        <v>1.2288396704547992</v>
+      </c>
+      <c r="U25">
+        <f t="shared" si="2"/>
+        <v>1.2271605524180154</v>
+      </c>
+      <c r="V25">
+        <f t="shared" si="3"/>
+        <v>1.2277354675261287</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>230</v>
+      </c>
+      <c r="B26" s="1">
         <v>10</v>
       </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25">
-        <v>230</v>
-      </c>
-      <c r="M25" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26">
-        <v>240</v>
-      </c>
-      <c r="B26" s="1">
-        <v>0</v>
-      </c>
       <c r="C26" s="1">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D26">
-        <v>-60</v>
+        <v>-70</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>1</v>
@@ -1556,30 +2255,60 @@
         <v>240</v>
       </c>
       <c r="J26">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K26">
         <v>0</v>
       </c>
       <c r="L26">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="M26" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N26">
+        <v>55888</v>
+      </c>
+      <c r="O26">
+        <v>246525</v>
+      </c>
+      <c r="P26">
+        <v>-302412</v>
+      </c>
+      <c r="Q26">
+        <v>45537</v>
+      </c>
+      <c r="R26">
+        <v>200803</v>
+      </c>
+      <c r="S26">
+        <v>-246341</v>
+      </c>
+      <c r="T26" s="1">
+        <f t="shared" si="5"/>
+        <v>1.2273096602762588</v>
+      </c>
+      <c r="U26">
+        <f t="shared" si="2"/>
+        <v>1.2276958013575494</v>
+      </c>
+      <c r="V26">
+        <f t="shared" si="3"/>
+        <v>1.2276153786823956</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="B27" s="1">
-        <v>-10</v>
-      </c>
-      <c r="C27">
-        <v>70</v>
-      </c>
-      <c r="D27" s="1">
-        <v>-50</v>
+        <v>0</v>
+      </c>
+      <c r="C27" s="1">
+        <v>60</v>
+      </c>
+      <c r="D27">
+        <v>-60</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>1</v>
@@ -1588,7 +2317,7 @@
         <v>7</v>
       </c>
       <c r="G27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H27">
         <v>0</v>
@@ -1597,30 +2326,60 @@
         <v>240</v>
       </c>
       <c r="J27">
-        <v>-10</v>
+        <v>0</v>
       </c>
       <c r="K27">
         <v>0</v>
       </c>
       <c r="L27">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="M27" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>278705</v>
+      </c>
+      <c r="P27">
+        <v>-278705</v>
+      </c>
+      <c r="Q27">
+        <v>0</v>
+      </c>
+      <c r="R27">
+        <v>227023</v>
+      </c>
+      <c r="S27">
+        <v>-227023</v>
+      </c>
+      <c r="T27" t="e">
+        <f t="shared" si="5"/>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U27">
+        <f t="shared" si="2"/>
+        <v>1.2276509428560103</v>
+      </c>
+      <c r="V27">
+        <f t="shared" si="3"/>
+        <v>1.2276509428560103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="B28" s="1">
-        <v>-20</v>
+        <v>-10</v>
       </c>
       <c r="C28">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="D28" s="1">
-        <v>-40</v>
+        <v>-50</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>1</v>
@@ -1632,36 +2391,66 @@
         <v>12</v>
       </c>
       <c r="H28">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I28">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="J28">
+        <v>-10</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>250</v>
+      </c>
+      <c r="M28" t="s">
+        <v>21</v>
+      </c>
+      <c r="N28">
+        <v>-55888</v>
+      </c>
+      <c r="O28">
+        <v>302412</v>
+      </c>
+      <c r="P28">
+        <v>-246525</v>
+      </c>
+      <c r="Q28">
+        <v>-45542</v>
+      </c>
+      <c r="R28">
+        <v>246342</v>
+      </c>
+      <c r="S28">
+        <v>-200800</v>
+      </c>
+      <c r="T28">
+        <f t="shared" si="5"/>
+        <v>1.2271749154626499</v>
+      </c>
+      <c r="U28">
+        <f t="shared" si="2"/>
+        <v>1.2276103953040893</v>
+      </c>
+      <c r="V28">
+        <f t="shared" si="3"/>
+        <v>1.2277141434262948</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>260</v>
+      </c>
+      <c r="B29" s="1">
+        <v>-20</v>
+      </c>
+      <c r="C29">
+        <v>80</v>
+      </c>
+      <c r="D29" s="1">
         <v>-40</v>
-      </c>
-      <c r="K28">
-        <v>1</v>
-      </c>
-      <c r="L28">
-        <v>260</v>
-      </c>
-      <c r="M28" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29">
-        <v>270</v>
-      </c>
-      <c r="B29" s="1">
-        <v>-30</v>
-      </c>
-      <c r="C29">
-        <v>90</v>
-      </c>
-      <c r="D29" s="1">
-        <v>-30</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>1</v>
@@ -1679,39 +2468,69 @@
         <v>300</v>
       </c>
       <c r="J29">
-        <v>-30</v>
+        <v>-40</v>
       </c>
       <c r="K29">
         <v>1</v>
       </c>
       <c r="L29">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="M29" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N29">
+        <v>-110077</v>
+      </c>
+      <c r="O29">
+        <v>316935</v>
+      </c>
+      <c r="P29">
+        <v>-206860</v>
+      </c>
+      <c r="Q29">
+        <v>-89563</v>
+      </c>
+      <c r="R29">
+        <v>258142</v>
+      </c>
+      <c r="S29">
+        <v>-168580</v>
+      </c>
+      <c r="T29">
+        <f t="shared" si="5"/>
+        <v>1.2290454763685896</v>
+      </c>
+      <c r="U29">
+        <f t="shared" si="2"/>
+        <v>1.227754491713863</v>
+      </c>
+      <c r="V29">
+        <f t="shared" si="3"/>
+        <v>1.2270731996678135</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="B30" s="1">
-        <v>-40</v>
+        <v>-30</v>
       </c>
       <c r="C30">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="D30" s="1">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H30">
         <v>2</v>
@@ -1720,30 +2539,60 @@
         <v>300</v>
       </c>
       <c r="J30">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="K30">
         <v>1</v>
       </c>
       <c r="L30">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="M30" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N30">
+        <v>-160920</v>
+      </c>
+      <c r="O30">
+        <v>321830</v>
+      </c>
+      <c r="P30">
+        <v>-160913</v>
+      </c>
+      <c r="Q30">
+        <v>-131006</v>
+      </c>
+      <c r="R30">
+        <v>262144</v>
+      </c>
+      <c r="S30">
+        <v>-131137</v>
+      </c>
+      <c r="T30">
+        <f t="shared" si="5"/>
+        <v>1.228340686686106</v>
+      </c>
+      <c r="U30">
+        <f t="shared" si="2"/>
+        <v>1.2276840209960938</v>
+      </c>
+      <c r="V30" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2270602499675911</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="B31" s="1">
-        <v>-50</v>
+        <v>-40</v>
       </c>
       <c r="C31">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="D31" s="1">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>2</v>
@@ -1761,30 +2610,60 @@
         <v>300</v>
       </c>
       <c r="J31">
+        <v>-20</v>
+      </c>
+      <c r="K31">
+        <v>1</v>
+      </c>
+      <c r="L31">
+        <v>280</v>
+      </c>
+      <c r="M31" t="s">
+        <v>23</v>
+      </c>
+      <c r="N31">
+        <v>-206868</v>
+      </c>
+      <c r="O31">
+        <v>316941</v>
+      </c>
+      <c r="P31">
+        <v>-110075</v>
+      </c>
+      <c r="Q31">
+        <v>-168460</v>
+      </c>
+      <c r="R31">
+        <v>258172</v>
+      </c>
+      <c r="S31">
+        <v>-89711</v>
+      </c>
+      <c r="T31">
+        <f t="shared" si="5"/>
+        <v>1.2279947762080019</v>
+      </c>
+      <c r="U31">
+        <f t="shared" si="2"/>
+        <v>1.2276350649954293</v>
+      </c>
+      <c r="V31" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2269955746786905</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>290</v>
+      </c>
+      <c r="B32" s="1">
+        <v>-50</v>
+      </c>
+      <c r="C32">
+        <v>70</v>
+      </c>
+      <c r="D32" s="1">
         <v>-10</v>
-      </c>
-      <c r="K31">
-        <v>1</v>
-      </c>
-      <c r="L31">
-        <v>290</v>
-      </c>
-      <c r="M31" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>300</v>
-      </c>
-      <c r="B32">
-        <v>-60</v>
-      </c>
-      <c r="C32" s="1">
-        <v>60</v>
-      </c>
-      <c r="D32" s="1">
-        <v>0</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>2</v>
@@ -1793,7 +2672,7 @@
         <v>10</v>
       </c>
       <c r="G32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H32">
         <v>2</v>
@@ -1802,30 +2681,60 @@
         <v>300</v>
       </c>
       <c r="J32">
-        <v>0</v>
+        <v>-10</v>
       </c>
       <c r="K32">
         <v>1</v>
       </c>
       <c r="L32">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="M32" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N32">
+        <v>-246534</v>
+      </c>
+      <c r="O32">
+        <v>302417</v>
+      </c>
+      <c r="P32">
+        <v>-55884</v>
+      </c>
+      <c r="Q32">
+        <v>-200800</v>
+      </c>
+      <c r="R32">
+        <v>246342</v>
+      </c>
+      <c r="S32">
+        <v>-45542</v>
+      </c>
+      <c r="T32">
+        <f t="shared" si="5"/>
+        <v>1.2277589641434263</v>
+      </c>
+      <c r="U32">
+        <f t="shared" si="2"/>
+        <v>1.2276306922895812</v>
+      </c>
+      <c r="V32" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2270870844495192</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="B33">
-        <v>-70</v>
+        <v>-60</v>
       </c>
       <c r="C33" s="1">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="D33" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>2</v>
@@ -1843,30 +2752,60 @@
         <v>300</v>
       </c>
       <c r="J33">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K33">
         <v>1</v>
       </c>
       <c r="L33">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="M33" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N33">
+        <v>-278713</v>
+      </c>
+      <c r="O33">
+        <v>278713</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33">
+        <v>-227023</v>
+      </c>
+      <c r="R33">
+        <v>227023</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <f t="shared" si="5"/>
+        <v>1.227686181576316</v>
+      </c>
+      <c r="U33">
+        <f t="shared" si="2"/>
+        <v>1.227686181576316</v>
+      </c>
+      <c r="V33" s="1" t="e">
+        <f t="shared" si="3"/>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="B34">
-        <v>-80</v>
+        <v>-70</v>
       </c>
       <c r="C34" s="1">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="D34" s="1">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>2</v>
@@ -1884,30 +2823,60 @@
         <v>300</v>
       </c>
       <c r="J34">
+        <v>10</v>
+      </c>
+      <c r="K34">
+        <v>1</v>
+      </c>
+      <c r="L34">
+        <v>310</v>
+      </c>
+      <c r="M34" t="s">
+        <v>21</v>
+      </c>
+      <c r="N34">
+        <v>-302417</v>
+      </c>
+      <c r="O34">
+        <v>246534</v>
+      </c>
+      <c r="P34">
+        <v>55884</v>
+      </c>
+      <c r="Q34">
+        <v>-246340</v>
+      </c>
+      <c r="R34">
+        <v>200802</v>
+      </c>
+      <c r="S34">
+        <v>45538</v>
+      </c>
+      <c r="T34">
+        <f t="shared" si="5"/>
+        <v>1.2276406592514411</v>
+      </c>
+      <c r="U34">
+        <f t="shared" si="2"/>
+        <v>1.2277467355902829</v>
+      </c>
+      <c r="V34" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2271948702182793</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>320</v>
+      </c>
+      <c r="B35">
+        <v>-80</v>
+      </c>
+      <c r="C35" s="1">
+        <v>40</v>
+      </c>
+      <c r="D35" s="1">
         <v>20</v>
-      </c>
-      <c r="K34">
-        <v>1</v>
-      </c>
-      <c r="L34">
-        <v>320</v>
-      </c>
-      <c r="M34" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>330</v>
-      </c>
-      <c r="B35">
-        <v>-90</v>
-      </c>
-      <c r="C35" s="1">
-        <v>30</v>
-      </c>
-      <c r="D35" s="1">
-        <v>30</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>2</v>
@@ -1925,39 +2894,69 @@
         <v>300</v>
       </c>
       <c r="J35">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="K35">
         <v>1</v>
       </c>
       <c r="L35">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="M35" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N35">
+        <v>-316941</v>
+      </c>
+      <c r="O35">
+        <v>206868</v>
+      </c>
+      <c r="P35">
+        <v>110075</v>
+      </c>
+      <c r="Q35">
+        <v>-258169</v>
+      </c>
+      <c r="R35">
+        <v>168465</v>
+      </c>
+      <c r="S35">
+        <v>89705</v>
+      </c>
+      <c r="T35">
+        <f t="shared" si="5"/>
+        <v>1.2276493304773231</v>
+      </c>
+      <c r="U35">
+        <f t="shared" si="2"/>
+        <v>1.2279583296233638</v>
+      </c>
+      <c r="V35" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2270776433866564</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="B36">
-        <v>-80</v>
+        <v>-90</v>
       </c>
       <c r="C36" s="1">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D36" s="1">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F36" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G36" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H36">
         <v>2</v>
@@ -1966,30 +2965,60 @@
         <v>300</v>
       </c>
       <c r="J36">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="K36">
         <v>1</v>
       </c>
       <c r="L36">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="M36" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N36">
+        <v>-321830</v>
+      </c>
+      <c r="O36">
+        <v>160920</v>
+      </c>
+      <c r="P36">
+        <v>160913</v>
+      </c>
+      <c r="Q36">
+        <v>-262143</v>
+      </c>
+      <c r="R36">
+        <v>131015</v>
+      </c>
+      <c r="S36">
+        <v>131129</v>
+      </c>
+      <c r="T36">
+        <f t="shared" si="5"/>
+        <v>1.227688704256837</v>
+      </c>
+      <c r="U36">
+        <f t="shared" si="2"/>
+        <v>1.2282563065297867</v>
+      </c>
+      <c r="V36" s="1">
+        <f t="shared" si="3"/>
+        <v>1.2271351112263496</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="B37">
-        <v>-70</v>
+        <v>-80</v>
       </c>
       <c r="C37" s="1">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D37" s="1">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>0</v>
@@ -2001,26 +3030,127 @@
         <v>11</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I37">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="J37">
+        <v>40</v>
+      </c>
+      <c r="K37">
+        <v>1</v>
+      </c>
+      <c r="L37">
+        <v>340</v>
+      </c>
+      <c r="M37" t="s">
+        <v>23</v>
+      </c>
+      <c r="N37">
+        <v>-316935</v>
+      </c>
+      <c r="O37">
+        <v>110077</v>
+      </c>
+      <c r="P37">
+        <v>206860</v>
+      </c>
+      <c r="Q37">
+        <v>-258146</v>
+      </c>
+      <c r="R37">
+        <v>89578</v>
+      </c>
+      <c r="S37">
+        <v>168568</v>
+      </c>
+      <c r="T37">
+        <f t="shared" si="5"/>
+        <v>1.2277354675261287</v>
+      </c>
+      <c r="U37" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2288396704547992</v>
+      </c>
+      <c r="V37">
+        <f t="shared" si="3"/>
+        <v>1.2271605524180154</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>350</v>
+      </c>
+      <c r="B38">
+        <v>-70</v>
+      </c>
+      <c r="C38" s="1">
         <v>10</v>
       </c>
-      <c r="K37">
-        <v>0</v>
-      </c>
-      <c r="L37">
+      <c r="D38" s="1">
+        <v>50</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F38" t="s">
+        <v>5</v>
+      </c>
+      <c r="G38" t="s">
+        <v>11</v>
+      </c>
+      <c r="H38">
+        <v>0</v>
+      </c>
+      <c r="I38">
+        <v>0</v>
+      </c>
+      <c r="J38">
+        <v>10</v>
+      </c>
+      <c r="K38">
+        <v>0</v>
+      </c>
+      <c r="L38">
         <v>350</v>
       </c>
-      <c r="M37" t="s">
+      <c r="M38" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="E38" s="1"/>
+      <c r="N38">
+        <v>-302412</v>
+      </c>
+      <c r="O38">
+        <v>55888</v>
+      </c>
+      <c r="P38">
+        <v>246525</v>
+      </c>
+      <c r="Q38">
+        <v>-246341</v>
+      </c>
+      <c r="R38">
+        <v>45537</v>
+      </c>
+      <c r="S38">
+        <v>200803</v>
+      </c>
+      <c r="T38">
+        <f t="shared" si="5"/>
+        <v>1.2276153786823956</v>
+      </c>
+      <c r="U38" s="1">
+        <f t="shared" si="2"/>
+        <v>1.2273096602762588</v>
+      </c>
+      <c r="V38">
+        <f t="shared" si="3"/>
+        <v>1.2276958013575494</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="E39" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Reduced angles to 16 bits.
</commit_message>
<xml_diff>
--- a/angle.xlsx
+++ b/angle.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\radio-zcu208\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110D5E8C-C0E4-4AFF-908B-3BC8D400B257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F6B65B7-04BC-4B54-802D-F30EBC541686}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2715" yWindow="5205" windowWidth="19140" windowHeight="10635" xr2:uid="{95DD9B03-E977-4F2B-8BD5-666F9F270815}"/>
+    <workbookView xWindow="2160" yWindow="4530" windowWidth="19140" windowHeight="10635" xr2:uid="{95DD9B03-E977-4F2B-8BD5-666F9F270815}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -643,17 +643,17 @@
         <v>278705</v>
       </c>
       <c r="Q3">
-        <v>-227023</v>
+        <v>-14188</v>
       </c>
       <c r="R3">
         <v>0</v>
       </c>
       <c r="S3">
-        <v>227023</v>
+        <v>14188</v>
       </c>
       <c r="T3">
         <f>N3/Q3</f>
-        <v>1.2276509428560103</v>
+        <v>19.643712996898788</v>
       </c>
       <c r="U3" s="1" t="e">
         <f>O3/R3</f>
@@ -661,7 +661,7 @@
       </c>
       <c r="V3">
         <f>P3/S3</f>
-        <v>1.2276509428560103</v>
+        <v>19.643712996898788</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
@@ -699,7 +699,7 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>10</v>
+        <v>10.01</v>
       </c>
       <c r="M4" t="s">
         <v>21</v>
@@ -714,25 +714,25 @@
         <v>302412</v>
       </c>
       <c r="Q4">
-        <v>-200800</v>
+        <v>-12550</v>
       </c>
       <c r="R4">
-        <v>-45542</v>
+        <v>-2847</v>
       </c>
       <c r="S4">
-        <v>246342</v>
+        <v>15396</v>
       </c>
       <c r="T4">
         <f t="shared" ref="T4:V4" si="0">N4/Q4</f>
-        <v>1.2277141434262948</v>
+        <v>19.643426294820717</v>
       </c>
       <c r="U4" s="1">
         <f t="shared" si="0"/>
-        <v>1.2271749154626499</v>
+        <v>19.630488233227958</v>
       </c>
       <c r="V4">
         <f t="shared" si="0"/>
-        <v>1.2276103953040893</v>
+        <v>19.642244738893218</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
@@ -770,7 +770,7 @@
         <v>1</v>
       </c>
       <c r="L5">
-        <v>20</v>
+        <v>19.98</v>
       </c>
       <c r="M5" t="s">
         <v>22</v>
@@ -785,25 +785,25 @@
         <v>316935</v>
       </c>
       <c r="Q5">
-        <v>-168579</v>
+        <v>-10536</v>
       </c>
       <c r="R5">
-        <v>-89565</v>
+        <v>-5599</v>
       </c>
       <c r="S5">
-        <v>258143</v>
+        <v>16134</v>
       </c>
       <c r="T5">
         <f t="shared" ref="T5" si="1">N5/Q5</f>
-        <v>1.2270804785886735</v>
+        <v>19.633637053910402</v>
       </c>
       <c r="U5" s="1">
         <f t="shared" ref="U5:U38" si="2">O5/R5</f>
-        <v>1.2290180315971642</v>
+        <v>19.660117878192533</v>
       </c>
       <c r="V5">
         <f t="shared" ref="V5:V38" si="3">P5/S5</f>
-        <v>1.2277497356116571</v>
+        <v>19.643919672740797</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
@@ -841,7 +841,7 @@
         <v>1</v>
       </c>
       <c r="L6">
-        <v>30</v>
+        <v>29.98</v>
       </c>
       <c r="M6" t="s">
         <v>22</v>
@@ -856,25 +856,25 @@
         <v>321803</v>
       </c>
       <c r="Q6">
-        <v>-131137</v>
+        <v>-8196</v>
       </c>
       <c r="R6">
-        <v>-131006</v>
+        <v>-8188</v>
       </c>
       <c r="S6">
-        <v>262144</v>
+        <v>16384</v>
       </c>
       <c r="T6" s="1">
         <f t="shared" ref="T6:T7" si="4">N6/Q6</f>
-        <v>1.2270602499675911</v>
+        <v>19.633113714006832</v>
       </c>
       <c r="U6">
         <f t="shared" si="2"/>
-        <v>1.228340686686106</v>
+        <v>19.653150952613579</v>
       </c>
       <c r="V6">
         <f t="shared" si="3"/>
-        <v>1.2275810241699219</v>
+        <v>19.64129638671875</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
@@ -912,7 +912,7 @@
         <v>1</v>
       </c>
       <c r="L7">
-        <v>40</v>
+        <v>39.979999999999997</v>
       </c>
       <c r="M7" t="s">
         <v>22</v>
@@ -927,25 +927,25 @@
         <v>316941</v>
       </c>
       <c r="Q7">
-        <v>-89711</v>
+        <v>-5609</v>
       </c>
       <c r="R7">
-        <v>-168460</v>
+        <v>-10526</v>
       </c>
       <c r="S7">
-        <v>258172</v>
+        <v>16136</v>
       </c>
       <c r="T7" s="1">
         <f t="shared" si="4"/>
-        <v>1.2269955746786905</v>
+        <v>19.624710287038688</v>
       </c>
       <c r="U7">
         <f t="shared" si="2"/>
-        <v>1.2279947762080019</v>
+        <v>19.653049591487743</v>
       </c>
       <c r="V7">
         <f t="shared" si="3"/>
-        <v>1.2276350649954293</v>
+        <v>19.64185671789787</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
@@ -983,7 +983,7 @@
         <v>1</v>
       </c>
       <c r="L8">
-        <v>50</v>
+        <v>49.99</v>
       </c>
       <c r="M8" t="s">
         <v>21</v>
@@ -998,25 +998,25 @@
         <v>302417</v>
       </c>
       <c r="Q8">
-        <v>-45542</v>
+        <v>-2847</v>
       </c>
       <c r="R8">
-        <v>-200800</v>
+        <v>-12549</v>
       </c>
       <c r="S8">
-        <v>246342</v>
+        <v>15397</v>
       </c>
       <c r="T8" s="1">
-        <f t="shared" ref="T8:V38" si="5">N8/Q8</f>
-        <v>1.2270870844495192</v>
+        <f t="shared" ref="T8:T38" si="5">N8/Q8</f>
+        <v>19.629083245521603</v>
       </c>
       <c r="U8">
         <f t="shared" si="2"/>
-        <v>1.2277589641434263</v>
+        <v>19.645708821420033</v>
       </c>
       <c r="V8">
         <f t="shared" si="3"/>
-        <v>1.2276306922895812</v>
+        <v>19.641293758524387</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
@@ -1072,10 +1072,10 @@
         <v>0</v>
       </c>
       <c r="R9">
-        <v>-227023</v>
+        <v>-14188</v>
       </c>
       <c r="S9">
-        <v>227023</v>
+        <v>14188</v>
       </c>
       <c r="T9" t="e">
         <f t="shared" si="5"/>
@@ -1083,11 +1083,11 @@
       </c>
       <c r="U9">
         <f t="shared" si="2"/>
-        <v>1.227686181576316</v>
+        <v>19.644276853679166</v>
       </c>
       <c r="V9">
         <f t="shared" si="3"/>
-        <v>1.227686181576316</v>
+        <v>19.644276853679166</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
@@ -1140,25 +1140,25 @@
         <v>246534</v>
       </c>
       <c r="Q10">
-        <v>45538</v>
+        <v>2846</v>
       </c>
       <c r="R10">
-        <v>-246340</v>
+        <v>-15396</v>
       </c>
       <c r="S10">
-        <v>200802</v>
+        <v>12550</v>
       </c>
       <c r="T10">
         <f t="shared" si="5"/>
-        <v>1.2271948702182793</v>
+        <v>19.635980323260718</v>
       </c>
       <c r="U10">
         <f t="shared" si="2"/>
-        <v>1.2276406592514411</v>
+        <v>19.642569498571056</v>
       </c>
       <c r="V10">
         <f t="shared" si="3"/>
-        <v>1.2277467355902829</v>
+        <v>19.644143426294821</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
@@ -1196,7 +1196,7 @@
         <v>1</v>
       </c>
       <c r="L11">
-        <v>80</v>
+        <v>80.010000000000005</v>
       </c>
       <c r="M11" t="s">
         <v>22</v>
@@ -1211,25 +1211,25 @@
         <v>206868</v>
       </c>
       <c r="Q11">
-        <v>89705</v>
+        <v>5606</v>
       </c>
       <c r="R11">
-        <v>-258169</v>
+        <v>-16135</v>
       </c>
       <c r="S11">
-        <v>168465</v>
+        <v>10529</v>
       </c>
       <c r="T11">
         <f t="shared" si="5"/>
-        <v>1.2270776433866564</v>
+        <v>19.635212272565109</v>
       </c>
       <c r="U11">
         <f t="shared" si="2"/>
-        <v>1.2276493304773231</v>
+        <v>19.643074062596838</v>
       </c>
       <c r="V11">
         <f t="shared" si="3"/>
-        <v>1.2279583296233638</v>
+        <v>19.647449900275429</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
@@ -1267,7 +1267,7 @@
         <v>1</v>
       </c>
       <c r="L12">
-        <v>90</v>
+        <v>90.01</v>
       </c>
       <c r="M12" t="s">
         <v>22</v>
@@ -1282,25 +1282,25 @@
         <v>160920</v>
       </c>
       <c r="Q12">
-        <v>131129</v>
+        <v>8194</v>
       </c>
       <c r="R12">
-        <v>-262143</v>
+        <v>-16384</v>
       </c>
       <c r="S12">
-        <v>131015</v>
+        <v>8190</v>
       </c>
       <c r="T12">
         <f t="shared" si="5"/>
-        <v>1.2271351112263496</v>
+        <v>19.637905784720527</v>
       </c>
       <c r="U12">
         <f t="shared" si="2"/>
-        <v>1.2275857070377618</v>
+        <v>19.64129638671875</v>
       </c>
       <c r="V12" s="1">
         <f t="shared" si="3"/>
-        <v>1.2282563065297867</v>
+        <v>19.64835164835165</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
@@ -1338,7 +1338,7 @@
         <v>1</v>
       </c>
       <c r="L13">
-        <v>100</v>
+        <v>100.01</v>
       </c>
       <c r="M13" t="s">
         <v>22</v>
@@ -1353,25 +1353,25 @@
         <v>110077</v>
       </c>
       <c r="Q13">
-        <v>168568</v>
+        <v>10534</v>
       </c>
       <c r="R13">
-        <v>-258146</v>
+        <v>-16134</v>
       </c>
       <c r="S13">
-        <v>89577</v>
+        <v>5600</v>
       </c>
       <c r="T13">
         <f t="shared" si="5"/>
-        <v>1.2271605524180154</v>
+        <v>19.637364723751663</v>
       </c>
       <c r="U13">
         <f t="shared" si="2"/>
-        <v>1.2277354675261287</v>
+        <v>19.643919672740797</v>
       </c>
       <c r="V13" s="1">
         <f t="shared" si="3"/>
-        <v>1.2288533887046897</v>
+        <v>19.656607142857144</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
@@ -1424,25 +1424,25 @@
         <v>55888</v>
       </c>
       <c r="Q14">
-        <v>200803</v>
+        <v>12550</v>
       </c>
       <c r="R14">
-        <v>-246341</v>
+        <v>-15396</v>
       </c>
       <c r="S14">
-        <v>45537</v>
+        <v>2846</v>
       </c>
       <c r="T14">
         <f t="shared" si="5"/>
-        <v>1.2276958013575494</v>
+        <v>19.643426294820717</v>
       </c>
       <c r="U14">
         <f t="shared" si="2"/>
-        <v>1.2276153786823956</v>
+        <v>19.642244738893218</v>
       </c>
       <c r="V14" s="1">
         <f t="shared" si="3"/>
-        <v>1.2273096602762588</v>
+        <v>19.63738580463809</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
@@ -1495,21 +1495,21 @@
         <v>0</v>
       </c>
       <c r="Q15">
-        <v>227023</v>
+        <v>14188</v>
       </c>
       <c r="R15">
-        <v>-227023</v>
+        <v>-14188</v>
       </c>
       <c r="S15">
         <v>0</v>
       </c>
       <c r="T15">
         <f t="shared" si="5"/>
-        <v>1.2276509428560103</v>
+        <v>19.643712996898788</v>
       </c>
       <c r="U15">
         <f t="shared" si="2"/>
-        <v>1.2276509428560103</v>
+        <v>19.643712996898788</v>
       </c>
       <c r="V15" s="1" t="e">
         <f t="shared" si="3"/>
@@ -1551,7 +1551,7 @@
         <v>0</v>
       </c>
       <c r="L16">
-        <v>130</v>
+        <v>130.01</v>
       </c>
       <c r="M16" t="s">
         <v>21</v>
@@ -1566,25 +1566,25 @@
         <v>-55888</v>
       </c>
       <c r="Q16">
-        <v>246342</v>
+        <v>15396</v>
       </c>
       <c r="R16">
-        <v>-200800</v>
+        <v>-12550</v>
       </c>
       <c r="S16">
-        <v>-45542</v>
+        <v>-2847</v>
       </c>
       <c r="T16">
         <f t="shared" si="5"/>
-        <v>1.2276103953040893</v>
+        <v>19.642244738893218</v>
       </c>
       <c r="U16">
         <f t="shared" si="2"/>
-        <v>1.2277141434262948</v>
+        <v>19.643426294820717</v>
       </c>
       <c r="V16" s="1">
         <f t="shared" si="3"/>
-        <v>1.2271749154626499</v>
+        <v>19.630488233227958</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
@@ -1622,7 +1622,7 @@
         <v>0</v>
       </c>
       <c r="L17">
-        <v>140</v>
+        <v>139.97999999999999</v>
       </c>
       <c r="M17" t="s">
         <v>24</v>
@@ -1637,25 +1637,25 @@
         <v>-110077</v>
       </c>
       <c r="Q17">
-        <v>258143</v>
+        <v>16134</v>
       </c>
       <c r="R17">
-        <v>-168579</v>
+        <v>-10536</v>
       </c>
       <c r="S17">
-        <v>-89565</v>
+        <v>-5599</v>
       </c>
       <c r="T17">
         <f t="shared" si="5"/>
-        <v>1.2277497356116571</v>
+        <v>19.643919672740797</v>
       </c>
       <c r="U17">
         <f t="shared" si="2"/>
-        <v>1.2270804785886735</v>
+        <v>19.633637053910402</v>
       </c>
       <c r="V17" s="1">
         <f t="shared" si="3"/>
-        <v>1.2290180315971642</v>
+        <v>19.660117878192533</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
@@ -1693,7 +1693,7 @@
         <v>1</v>
       </c>
       <c r="L18">
-        <v>150</v>
+        <v>149.97999999999999</v>
       </c>
       <c r="M18" t="s">
         <v>24</v>
@@ -1708,25 +1708,25 @@
         <v>-160920</v>
       </c>
       <c r="Q18">
-        <v>262144</v>
+        <v>16384</v>
       </c>
       <c r="R18">
-        <v>-131137</v>
+        <v>-8196</v>
       </c>
       <c r="S18">
-        <v>-131006</v>
+        <v>-8188</v>
       </c>
       <c r="T18">
         <f t="shared" si="5"/>
-        <v>1.2275810241699219</v>
+        <v>19.64129638671875</v>
       </c>
       <c r="U18" s="1">
         <f t="shared" si="2"/>
-        <v>1.2270602499675911</v>
+        <v>19.633113714006832</v>
       </c>
       <c r="V18">
         <f t="shared" si="3"/>
-        <v>1.228340686686106</v>
+        <v>19.653150952613579</v>
       </c>
     </row>
     <row r="19" spans="1:22" x14ac:dyDescent="0.25">
@@ -1764,7 +1764,7 @@
         <v>1</v>
       </c>
       <c r="L19">
-        <v>160</v>
+        <v>159.97999999999999</v>
       </c>
       <c r="M19" t="s">
         <v>24</v>
@@ -1779,25 +1779,25 @@
         <v>-206868</v>
       </c>
       <c r="Q19">
-        <v>258172</v>
+        <v>16136</v>
       </c>
       <c r="R19">
-        <v>-89711</v>
+        <v>-5609</v>
       </c>
       <c r="S19">
-        <v>-168460</v>
+        <v>-10526</v>
       </c>
       <c r="T19">
         <f t="shared" si="5"/>
-        <v>1.2276350649954293</v>
+        <v>19.64185671789787</v>
       </c>
       <c r="U19" s="1">
         <f t="shared" si="2"/>
-        <v>1.2269955746786905</v>
+        <v>19.624710287038688</v>
       </c>
       <c r="V19">
         <f t="shared" si="3"/>
-        <v>1.2279947762080019</v>
+        <v>19.653049591487743</v>
       </c>
     </row>
     <row r="20" spans="1:22" x14ac:dyDescent="0.25">
@@ -1835,7 +1835,7 @@
         <v>1</v>
       </c>
       <c r="L20">
-        <v>170</v>
+        <v>169.99</v>
       </c>
       <c r="M20" t="s">
         <v>21</v>
@@ -1850,25 +1850,25 @@
         <v>-246534</v>
       </c>
       <c r="Q20">
-        <v>246342</v>
+        <v>15397</v>
       </c>
       <c r="R20">
-        <v>-45542</v>
+        <v>-2847</v>
       </c>
       <c r="S20">
-        <v>-200800</v>
+        <v>-12549</v>
       </c>
       <c r="T20">
         <f t="shared" si="5"/>
-        <v>1.2276306922895812</v>
+        <v>19.641293758524387</v>
       </c>
       <c r="U20" s="1">
         <f t="shared" si="2"/>
-        <v>1.2270870844495192</v>
+        <v>19.629083245521603</v>
       </c>
       <c r="V20">
         <f t="shared" si="3"/>
-        <v>1.2277589641434263</v>
+        <v>19.645708821420033</v>
       </c>
     </row>
     <row r="21" spans="1:22" x14ac:dyDescent="0.25">
@@ -1921,17 +1921,17 @@
         <v>-278713</v>
       </c>
       <c r="Q21">
-        <v>227023</v>
+        <v>14188</v>
       </c>
       <c r="R21">
         <v>0</v>
       </c>
       <c r="S21">
-        <v>-227023</v>
+        <v>-14188</v>
       </c>
       <c r="T21">
         <f t="shared" si="5"/>
-        <v>1.227686181576316</v>
+        <v>19.644276853679166</v>
       </c>
       <c r="U21" s="1" t="e">
         <f t="shared" si="2"/>
@@ -1939,7 +1939,7 @@
       </c>
       <c r="V21">
         <f t="shared" si="3"/>
-        <v>1.227686181576316</v>
+        <v>19.644276853679166</v>
       </c>
     </row>
     <row r="22" spans="1:22" x14ac:dyDescent="0.25">
@@ -1992,25 +1992,25 @@
         <v>-302417</v>
       </c>
       <c r="Q22">
-        <v>200802</v>
+        <v>12550</v>
       </c>
       <c r="R22">
-        <v>45538</v>
+        <v>2846</v>
       </c>
       <c r="S22">
-        <v>-246340</v>
+        <v>-15396</v>
       </c>
       <c r="T22">
         <f t="shared" si="5"/>
-        <v>1.2277467355902829</v>
+        <v>19.644143426294821</v>
       </c>
       <c r="U22" s="1">
         <f t="shared" si="2"/>
-        <v>1.2271948702182793</v>
+        <v>19.635980323260718</v>
       </c>
       <c r="V22">
         <f t="shared" si="3"/>
-        <v>1.2276406592514411</v>
+        <v>19.642569498571056</v>
       </c>
     </row>
     <row r="23" spans="1:22" x14ac:dyDescent="0.25">
@@ -2063,25 +2063,25 @@
         <v>-316941</v>
       </c>
       <c r="Q23">
-        <v>168465</v>
+        <v>10529</v>
       </c>
       <c r="R23">
-        <v>89705</v>
+        <v>5606</v>
       </c>
       <c r="S23">
-        <v>-258169</v>
+        <v>-16135</v>
       </c>
       <c r="T23">
         <f t="shared" si="5"/>
-        <v>1.2279583296233638</v>
+        <v>19.647449900275429</v>
       </c>
       <c r="U23" s="1">
         <f t="shared" si="2"/>
-        <v>1.2270776433866564</v>
+        <v>19.635212272565109</v>
       </c>
       <c r="V23">
         <f t="shared" si="3"/>
-        <v>1.2276493304773231</v>
+        <v>19.643074062596838</v>
       </c>
     </row>
     <row r="24" spans="1:22" x14ac:dyDescent="0.25">
@@ -2119,7 +2119,7 @@
         <v>1</v>
       </c>
       <c r="L24">
-        <v>210</v>
+        <v>210.01</v>
       </c>
       <c r="M24" t="s">
         <v>24</v>
@@ -2134,25 +2134,25 @@
         <v>-321830</v>
       </c>
       <c r="Q24">
-        <v>131015</v>
+        <v>8190</v>
       </c>
       <c r="R24">
-        <v>131129</v>
+        <v>8194</v>
       </c>
       <c r="S24">
-        <v>-262143</v>
+        <v>-16384</v>
       </c>
       <c r="T24">
         <f t="shared" si="5"/>
-        <v>1.2282563065297867</v>
+        <v>19.64835164835165</v>
       </c>
       <c r="U24" s="1">
         <f t="shared" si="2"/>
-        <v>1.2271351112263496</v>
+        <v>19.637905784720527</v>
       </c>
       <c r="V24">
         <f t="shared" si="3"/>
-        <v>1.227688704256837</v>
+        <v>19.6429443359375</v>
       </c>
     </row>
     <row r="25" spans="1:22" x14ac:dyDescent="0.25">
@@ -2190,7 +2190,7 @@
         <v>1</v>
       </c>
       <c r="L25">
-        <v>220</v>
+        <v>220.01</v>
       </c>
       <c r="M25" t="s">
         <v>24</v>
@@ -2205,25 +2205,25 @@
         <v>-316935</v>
       </c>
       <c r="Q25">
-        <v>89578</v>
+        <v>5601</v>
       </c>
       <c r="R25">
-        <v>168568</v>
+        <v>10533</v>
       </c>
       <c r="S25">
-        <v>-258146</v>
+        <v>-16135</v>
       </c>
       <c r="T25" s="1">
         <f t="shared" si="5"/>
-        <v>1.2288396704547992</v>
+        <v>19.653097661131941</v>
       </c>
       <c r="U25">
         <f t="shared" si="2"/>
-        <v>1.2271605524180154</v>
+        <v>19.63922908952815</v>
       </c>
       <c r="V25">
         <f t="shared" si="3"/>
-        <v>1.2277354675261287</v>
+        <v>19.64270220018593</v>
       </c>
     </row>
     <row r="26" spans="1:22" x14ac:dyDescent="0.25">
@@ -2276,25 +2276,25 @@
         <v>-302412</v>
       </c>
       <c r="Q26">
-        <v>45537</v>
+        <v>2846</v>
       </c>
       <c r="R26">
-        <v>200803</v>
+        <v>12550</v>
       </c>
       <c r="S26">
-        <v>-246341</v>
+        <v>-15396</v>
       </c>
       <c r="T26" s="1">
         <f t="shared" si="5"/>
-        <v>1.2273096602762588</v>
+        <v>19.63738580463809</v>
       </c>
       <c r="U26">
         <f t="shared" si="2"/>
-        <v>1.2276958013575494</v>
+        <v>19.643426294820717</v>
       </c>
       <c r="V26">
         <f t="shared" si="3"/>
-        <v>1.2276153786823956</v>
+        <v>19.642244738893218</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.25">
@@ -2350,10 +2350,10 @@
         <v>0</v>
       </c>
       <c r="R27">
-        <v>227023</v>
+        <v>14188</v>
       </c>
       <c r="S27">
-        <v>-227023</v>
+        <v>-14188</v>
       </c>
       <c r="T27" t="e">
         <f t="shared" si="5"/>
@@ -2361,11 +2361,11 @@
       </c>
       <c r="U27">
         <f t="shared" si="2"/>
-        <v>1.2276509428560103</v>
+        <v>19.643712996898788</v>
       </c>
       <c r="V27">
         <f t="shared" si="3"/>
-        <v>1.2276509428560103</v>
+        <v>19.643712996898788</v>
       </c>
     </row>
     <row r="28" spans="1:22" x14ac:dyDescent="0.25">
@@ -2403,7 +2403,7 @@
         <v>0</v>
       </c>
       <c r="L28">
-        <v>250</v>
+        <v>250.01</v>
       </c>
       <c r="M28" t="s">
         <v>21</v>
@@ -2418,25 +2418,25 @@
         <v>-246525</v>
       </c>
       <c r="Q28">
-        <v>-45542</v>
+        <v>-2847</v>
       </c>
       <c r="R28">
-        <v>246342</v>
+        <v>15396</v>
       </c>
       <c r="S28">
-        <v>-200800</v>
+        <v>-12550</v>
       </c>
       <c r="T28">
         <f t="shared" si="5"/>
-        <v>1.2271749154626499</v>
+        <v>19.630488233227958</v>
       </c>
       <c r="U28">
         <f t="shared" si="2"/>
-        <v>1.2276103953040893</v>
+        <v>19.642244738893218</v>
       </c>
       <c r="V28">
         <f t="shared" si="3"/>
-        <v>1.2277141434262948</v>
+        <v>19.643426294820717</v>
       </c>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.25">
@@ -2474,7 +2474,7 @@
         <v>1</v>
       </c>
       <c r="L29">
-        <v>260</v>
+        <v>259.97000000000003</v>
       </c>
       <c r="M29" t="s">
         <v>23</v>
@@ -2489,25 +2489,25 @@
         <v>-206860</v>
       </c>
       <c r="Q29">
-        <v>-89563</v>
+        <v>-5598</v>
       </c>
       <c r="R29">
-        <v>258142</v>
+        <v>16134</v>
       </c>
       <c r="S29">
-        <v>-168580</v>
+        <v>-10536</v>
       </c>
       <c r="T29">
         <f t="shared" si="5"/>
-        <v>1.2290454763685896</v>
+        <v>19.663629867809931</v>
       </c>
       <c r="U29">
         <f t="shared" si="2"/>
-        <v>1.227754491713863</v>
+        <v>19.643919672740797</v>
       </c>
       <c r="V29">
         <f t="shared" si="3"/>
-        <v>1.2270731996678135</v>
+        <v>19.633637053910402</v>
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.25">
@@ -2545,7 +2545,7 @@
         <v>1</v>
       </c>
       <c r="L30">
-        <v>270</v>
+        <v>269.98</v>
       </c>
       <c r="M30" t="s">
         <v>23</v>
@@ -2560,25 +2560,25 @@
         <v>-160913</v>
       </c>
       <c r="Q30">
-        <v>-131006</v>
+        <v>-8186</v>
       </c>
       <c r="R30">
-        <v>262144</v>
+        <v>16383</v>
       </c>
       <c r="S30">
-        <v>-131137</v>
+        <v>-8197</v>
       </c>
       <c r="T30">
         <f t="shared" si="5"/>
-        <v>1.228340686686106</v>
+        <v>19.657952602003419</v>
       </c>
       <c r="U30">
         <f t="shared" si="2"/>
-        <v>1.2276840209960938</v>
+        <v>19.64414331929439</v>
       </c>
       <c r="V30" s="1">
         <f t="shared" si="3"/>
-        <v>1.2270602499675911</v>
+        <v>19.630718555569111</v>
       </c>
     </row>
     <row r="31" spans="1:22" x14ac:dyDescent="0.25">
@@ -2616,7 +2616,7 @@
         <v>1</v>
       </c>
       <c r="L31">
-        <v>280</v>
+        <v>279.98</v>
       </c>
       <c r="M31" t="s">
         <v>23</v>
@@ -2631,25 +2631,25 @@
         <v>-110075</v>
       </c>
       <c r="Q31">
-        <v>-168460</v>
+        <v>-10526</v>
       </c>
       <c r="R31">
-        <v>258172</v>
+        <v>16136</v>
       </c>
       <c r="S31">
-        <v>-89711</v>
+        <v>-5609</v>
       </c>
       <c r="T31">
         <f t="shared" si="5"/>
-        <v>1.2279947762080019</v>
+        <v>19.653049591487743</v>
       </c>
       <c r="U31">
         <f t="shared" si="2"/>
-        <v>1.2276350649954293</v>
+        <v>19.64185671789787</v>
       </c>
       <c r="V31" s="1">
         <f t="shared" si="3"/>
-        <v>1.2269955746786905</v>
+        <v>19.624710287038688</v>
       </c>
     </row>
     <row r="32" spans="1:22" x14ac:dyDescent="0.25">
@@ -2687,7 +2687,7 @@
         <v>1</v>
       </c>
       <c r="L32">
-        <v>290</v>
+        <v>289.99</v>
       </c>
       <c r="M32" t="s">
         <v>21</v>
@@ -2702,25 +2702,25 @@
         <v>-55884</v>
       </c>
       <c r="Q32">
-        <v>-200800</v>
+        <v>-12549</v>
       </c>
       <c r="R32">
-        <v>246342</v>
+        <v>15397</v>
       </c>
       <c r="S32">
-        <v>-45542</v>
+        <v>-2847</v>
       </c>
       <c r="T32">
         <f t="shared" si="5"/>
-        <v>1.2277589641434263</v>
+        <v>19.645708821420033</v>
       </c>
       <c r="U32">
         <f t="shared" si="2"/>
-        <v>1.2276306922895812</v>
+        <v>19.641293758524387</v>
       </c>
       <c r="V32" s="1">
         <f t="shared" si="3"/>
-        <v>1.2270870844495192</v>
+        <v>19.629083245521603</v>
       </c>
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.25">
@@ -2773,21 +2773,21 @@
         <v>0</v>
       </c>
       <c r="Q33">
-        <v>-227023</v>
+        <v>-14188</v>
       </c>
       <c r="R33">
-        <v>227023</v>
+        <v>14188</v>
       </c>
       <c r="S33">
         <v>0</v>
       </c>
       <c r="T33">
         <f t="shared" si="5"/>
-        <v>1.227686181576316</v>
+        <v>19.644276853679166</v>
       </c>
       <c r="U33">
         <f t="shared" si="2"/>
-        <v>1.227686181576316</v>
+        <v>19.644276853679166</v>
       </c>
       <c r="V33" s="1" t="e">
         <f t="shared" si="3"/>
@@ -2844,25 +2844,25 @@
         <v>55884</v>
       </c>
       <c r="Q34">
-        <v>-246340</v>
+        <v>-15396</v>
       </c>
       <c r="R34">
-        <v>200802</v>
+        <v>12550</v>
       </c>
       <c r="S34">
-        <v>45538</v>
+        <v>2846</v>
       </c>
       <c r="T34">
         <f t="shared" si="5"/>
-        <v>1.2276406592514411</v>
+        <v>19.642569498571056</v>
       </c>
       <c r="U34">
         <f t="shared" si="2"/>
-        <v>1.2277467355902829</v>
+        <v>19.644143426294821</v>
       </c>
       <c r="V34" s="1">
         <f t="shared" si="3"/>
-        <v>1.2271948702182793</v>
+        <v>19.635980323260718</v>
       </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.25">
@@ -2915,25 +2915,25 @@
         <v>110075</v>
       </c>
       <c r="Q35">
-        <v>-258169</v>
+        <v>-16135</v>
       </c>
       <c r="R35">
-        <v>168465</v>
+        <v>10529</v>
       </c>
       <c r="S35">
-        <v>89705</v>
+        <v>5606</v>
       </c>
       <c r="T35">
         <f t="shared" si="5"/>
-        <v>1.2276493304773231</v>
+        <v>19.643074062596838</v>
       </c>
       <c r="U35">
         <f t="shared" si="2"/>
-        <v>1.2279583296233638</v>
+        <v>19.647449900275429</v>
       </c>
       <c r="V35" s="1">
         <f t="shared" si="3"/>
-        <v>1.2270776433866564</v>
+        <v>19.635212272565109</v>
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.25">
@@ -2971,7 +2971,7 @@
         <v>1</v>
       </c>
       <c r="L36">
-        <v>330</v>
+        <v>330.01</v>
       </c>
       <c r="M36" t="s">
         <v>23</v>
@@ -2986,25 +2986,25 @@
         <v>160913</v>
       </c>
       <c r="Q36">
-        <v>-262143</v>
+        <v>-16384</v>
       </c>
       <c r="R36">
-        <v>131015</v>
+        <v>8190</v>
       </c>
       <c r="S36">
-        <v>131129</v>
+        <v>8194</v>
       </c>
       <c r="T36">
         <f t="shared" si="5"/>
-        <v>1.227688704256837</v>
+        <v>19.6429443359375</v>
       </c>
       <c r="U36">
         <f t="shared" si="2"/>
-        <v>1.2282563065297867</v>
+        <v>19.64835164835165</v>
       </c>
       <c r="V36" s="1">
         <f t="shared" si="3"/>
-        <v>1.2271351112263496</v>
+        <v>19.637905784720527</v>
       </c>
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.25">
@@ -3042,7 +3042,7 @@
         <v>1</v>
       </c>
       <c r="L37">
-        <v>340</v>
+        <v>340.01</v>
       </c>
       <c r="M37" t="s">
         <v>23</v>
@@ -3057,25 +3057,25 @@
         <v>206860</v>
       </c>
       <c r="Q37">
-        <v>-258146</v>
+        <v>-16135</v>
       </c>
       <c r="R37">
-        <v>89578</v>
+        <v>5601</v>
       </c>
       <c r="S37">
-        <v>168568</v>
+        <v>10533</v>
       </c>
       <c r="T37">
         <f t="shared" si="5"/>
-        <v>1.2277354675261287</v>
+        <v>19.64270220018593</v>
       </c>
       <c r="U37" s="1">
         <f t="shared" si="2"/>
-        <v>1.2288396704547992</v>
+        <v>19.653097661131941</v>
       </c>
       <c r="V37">
         <f t="shared" si="3"/>
-        <v>1.2271605524180154</v>
+        <v>19.63922908952815</v>
       </c>
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.25">
@@ -3128,25 +3128,25 @@
         <v>246525</v>
       </c>
       <c r="Q38">
-        <v>-246341</v>
+        <v>-15396</v>
       </c>
       <c r="R38">
-        <v>45537</v>
+        <v>2846</v>
       </c>
       <c r="S38">
-        <v>200803</v>
+        <v>12550</v>
       </c>
       <c r="T38">
         <f t="shared" si="5"/>
-        <v>1.2276153786823956</v>
+        <v>19.642244738893218</v>
       </c>
       <c r="U38" s="1">
         <f t="shared" si="2"/>
-        <v>1.2273096602762588</v>
+        <v>19.63738580463809</v>
       </c>
       <c r="V38">
         <f t="shared" si="3"/>
-        <v>1.2276958013575494</v>
+        <v>19.643426294820717</v>
       </c>
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.25">

</xml_diff>